<commit_message>
Autualizando preço e removendo promoções 27/03
</commit_message>
<xml_diff>
--- a/scripts/produtos.xlsx
+++ b/scripts/produtos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ListProducts\scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B9D2AA2-CBA8-4EC8-B42D-D03CF6AD9BD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9E36288-30CA-47D6-85F5-EDA6E990FC37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5116,51 +5116,6 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="4"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -5178,6 +5133,12 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -5187,7 +5148,43 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="4"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -5202,11 +5199,14 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -5227,10 +5227,10 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -5552,83 +5552,83 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="20.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="124" t="s">
+      <c r="A1" s="105" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="125"/>
-      <c r="C1" s="125"/>
-      <c r="D1" s="125"/>
-      <c r="E1" s="126"/>
+      <c r="B1" s="106"/>
+      <c r="C1" s="106"/>
+      <c r="D1" s="106"/>
+      <c r="E1" s="107"/>
     </row>
     <row r="2" spans="1:5" ht="20.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="129" t="s">
+      <c r="A2" s="112" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="103"/>
-      <c r="C2" s="103"/>
-      <c r="D2" s="104"/>
-      <c r="E2" s="128"/>
+      <c r="B2" s="109"/>
+      <c r="C2" s="109"/>
+      <c r="D2" s="110"/>
+      <c r="E2" s="111"/>
     </row>
     <row r="3" spans="1:5" ht="20.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="127" t="s">
+      <c r="A3" s="108" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="103"/>
-      <c r="C3" s="103"/>
-      <c r="D3" s="104"/>
-      <c r="E3" s="128"/>
+      <c r="B3" s="109"/>
+      <c r="C3" s="109"/>
+      <c r="D3" s="110"/>
+      <c r="E3" s="111"/>
     </row>
     <row r="4" spans="1:5" ht="20.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="127" t="s">
+      <c r="A4" s="108" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="103"/>
-      <c r="C4" s="103"/>
-      <c r="D4" s="104"/>
-      <c r="E4" s="128"/>
+      <c r="B4" s="109"/>
+      <c r="C4" s="109"/>
+      <c r="D4" s="110"/>
+      <c r="E4" s="111"/>
     </row>
     <row r="5" spans="1:5" ht="20.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="127" t="s">
+      <c r="A5" s="108" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="103"/>
-      <c r="C5" s="103"/>
-      <c r="D5" s="104"/>
-      <c r="E5" s="128"/>
+      <c r="B5" s="109"/>
+      <c r="C5" s="109"/>
+      <c r="D5" s="110"/>
+      <c r="E5" s="111"/>
     </row>
     <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="127"/>
-      <c r="B6" s="103"/>
-      <c r="C6" s="103"/>
-      <c r="D6" s="104"/>
-      <c r="E6" s="128"/>
+      <c r="A6" s="108"/>
+      <c r="B6" s="109"/>
+      <c r="C6" s="109"/>
+      <c r="D6" s="110"/>
+      <c r="E6" s="111"/>
     </row>
     <row r="7" spans="1:5" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="130" t="s">
+      <c r="A7" s="113" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="131"/>
-      <c r="C7" s="131"/>
-      <c r="D7" s="131"/>
-      <c r="E7" s="132"/>
+      <c r="B7" s="114"/>
+      <c r="C7" s="114"/>
+      <c r="D7" s="114"/>
+      <c r="E7" s="115"/>
     </row>
     <row r="8" spans="1:5" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="115" t="s">
+      <c r="A8" s="123" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="116"/>
-      <c r="C8" s="116"/>
-      <c r="D8" s="116"/>
-      <c r="E8" s="117"/>
+      <c r="B8" s="124"/>
+      <c r="C8" s="124"/>
+      <c r="D8" s="124"/>
+      <c r="E8" s="125"/>
     </row>
     <row r="9" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="118" t="s">
+      <c r="A9" s="122" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="112"/>
-      <c r="C9" s="112"/>
-      <c r="D9" s="112"/>
-      <c r="E9" s="113"/>
+      <c r="B9" s="119"/>
+      <c r="C9" s="119"/>
+      <c r="D9" s="119"/>
+      <c r="E9" s="120"/>
     </row>
     <row r="10" spans="1:5" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="66" t="s">
@@ -6239,7 +6239,7 @@
         <v>34</v>
       </c>
       <c r="E45" s="49">
-        <v>550</v>
+        <v>490</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -6256,7 +6256,7 @@
         <v>20</v>
       </c>
       <c r="E46" s="41">
-        <v>112</v>
+        <v>100</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -7314,20 +7314,20 @@
       </c>
     </row>
     <row r="109" spans="1:5" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A109" s="102"/>
-      <c r="B109" s="103"/>
-      <c r="C109" s="103"/>
-      <c r="D109" s="104"/>
-      <c r="E109" s="105"/>
+      <c r="A109" s="121"/>
+      <c r="B109" s="109"/>
+      <c r="C109" s="109"/>
+      <c r="D109" s="110"/>
+      <c r="E109" s="117"/>
     </row>
     <row r="110" spans="1:5" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A110" s="118" t="s">
+      <c r="A110" s="122" t="s">
         <v>86</v>
       </c>
-      <c r="B110" s="112"/>
-      <c r="C110" s="112"/>
-      <c r="D110" s="112"/>
-      <c r="E110" s="113"/>
+      <c r="B110" s="119"/>
+      <c r="C110" s="119"/>
+      <c r="D110" s="119"/>
+      <c r="E110" s="120"/>
     </row>
     <row r="111" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" s="66" t="s">
@@ -7619,20 +7619,20 @@
       </c>
     </row>
     <row r="128" spans="1:5" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A128" s="102"/>
-      <c r="B128" s="103"/>
-      <c r="C128" s="103"/>
-      <c r="D128" s="104"/>
-      <c r="E128" s="105"/>
+      <c r="A128" s="121"/>
+      <c r="B128" s="109"/>
+      <c r="C128" s="109"/>
+      <c r="D128" s="110"/>
+      <c r="E128" s="117"/>
     </row>
     <row r="129" spans="1:5" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A129" s="118" t="s">
+      <c r="A129" s="122" t="s">
         <v>95</v>
       </c>
-      <c r="B129" s="112"/>
-      <c r="C129" s="112"/>
-      <c r="D129" s="112"/>
-      <c r="E129" s="113"/>
+      <c r="B129" s="119"/>
+      <c r="C129" s="119"/>
+      <c r="D129" s="119"/>
+      <c r="E129" s="120"/>
     </row>
     <row r="130" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A130" s="66" t="s">
@@ -7788,20 +7788,20 @@
       </c>
     </row>
     <row r="139" spans="1:5" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A139" s="102"/>
-      <c r="B139" s="103"/>
-      <c r="C139" s="103"/>
-      <c r="D139" s="104"/>
-      <c r="E139" s="105"/>
+      <c r="A139" s="121"/>
+      <c r="B139" s="109"/>
+      <c r="C139" s="109"/>
+      <c r="D139" s="110"/>
+      <c r="E139" s="117"/>
     </row>
     <row r="140" spans="1:5" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A140" s="119" t="s">
+      <c r="A140" s="126" t="s">
         <v>106</v>
       </c>
-      <c r="B140" s="112"/>
-      <c r="C140" s="112"/>
-      <c r="D140" s="112"/>
-      <c r="E140" s="120"/>
+      <c r="B140" s="119"/>
+      <c r="C140" s="119"/>
+      <c r="D140" s="119"/>
+      <c r="E140" s="127"/>
     </row>
     <row r="141" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A141" s="66" t="s">
@@ -9045,20 +9045,20 @@
       </c>
     </row>
     <row r="214" spans="1:5" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A214" s="102"/>
-      <c r="B214" s="103"/>
-      <c r="C214" s="103"/>
-      <c r="D214" s="104"/>
-      <c r="E214" s="105"/>
+      <c r="A214" s="121"/>
+      <c r="B214" s="109"/>
+      <c r="C214" s="109"/>
+      <c r="D214" s="110"/>
+      <c r="E214" s="117"/>
     </row>
     <row r="215" spans="1:5" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A215" s="118" t="s">
+      <c r="A215" s="122" t="s">
         <v>148</v>
       </c>
-      <c r="B215" s="112"/>
-      <c r="C215" s="112"/>
-      <c r="D215" s="112"/>
-      <c r="E215" s="113"/>
+      <c r="B215" s="119"/>
+      <c r="C215" s="119"/>
+      <c r="D215" s="119"/>
+      <c r="E215" s="120"/>
     </row>
     <row r="216" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A216" s="66" t="s">
@@ -10266,20 +10266,20 @@
       </c>
     </row>
     <row r="287" spans="1:5" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A287" s="114"/>
-      <c r="B287" s="103"/>
-      <c r="C287" s="103"/>
-      <c r="D287" s="104"/>
-      <c r="E287" s="105"/>
+      <c r="A287" s="116"/>
+      <c r="B287" s="109"/>
+      <c r="C287" s="109"/>
+      <c r="D287" s="110"/>
+      <c r="E287" s="117"/>
     </row>
     <row r="288" spans="1:5" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A288" s="118" t="s">
+      <c r="A288" s="122" t="s">
         <v>186</v>
       </c>
-      <c r="B288" s="112"/>
-      <c r="C288" s="112"/>
-      <c r="D288" s="112"/>
-      <c r="E288" s="113"/>
+      <c r="B288" s="119"/>
+      <c r="C288" s="119"/>
+      <c r="D288" s="119"/>
+      <c r="E288" s="120"/>
     </row>
     <row r="289" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A289" s="66" t="s">
@@ -10548,7 +10548,7 @@
         <v>84</v>
       </c>
       <c r="E304" s="40">
-        <v>162.5</v>
+        <v>148</v>
       </c>
     </row>
     <row r="305" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -10565,7 +10565,7 @@
         <v>84</v>
       </c>
       <c r="E305" s="40">
-        <v>295</v>
+        <v>268.5</v>
       </c>
     </row>
     <row r="306" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -10582,7 +10582,7 @@
         <v>84</v>
       </c>
       <c r="E306" s="40">
-        <v>34.5</v>
+        <v>31.5</v>
       </c>
     </row>
     <row r="307" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -10871,7 +10871,7 @@
         <v>34</v>
       </c>
       <c r="E323" s="40">
-        <v>420</v>
+        <v>356</v>
       </c>
     </row>
     <row r="324" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -10888,7 +10888,7 @@
         <v>34</v>
       </c>
       <c r="E324" s="40">
-        <v>210</v>
+        <v>178</v>
       </c>
     </row>
     <row r="325" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -10905,7 +10905,7 @@
         <v>20</v>
       </c>
       <c r="E325" s="40">
-        <v>44</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="326" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -11534,7 +11534,7 @@
         <v>84</v>
       </c>
       <c r="E362" s="40">
-        <v>199.5</v>
+        <v>187.5</v>
       </c>
     </row>
     <row r="363" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -11551,7 +11551,7 @@
         <v>34</v>
       </c>
       <c r="E363" s="40">
-        <v>399</v>
+        <v>375</v>
       </c>
     </row>
     <row r="364" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -11568,7 +11568,7 @@
         <v>49</v>
       </c>
       <c r="E364" s="50">
-        <v>46</v>
+        <v>43.5</v>
       </c>
     </row>
     <row r="365" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -11844,20 +11844,20 @@
       </c>
     </row>
     <row r="381" spans="1:5" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A381" s="114"/>
-      <c r="B381" s="103"/>
-      <c r="C381" s="103"/>
-      <c r="D381" s="104"/>
-      <c r="E381" s="105"/>
+      <c r="A381" s="116"/>
+      <c r="B381" s="109"/>
+      <c r="C381" s="109"/>
+      <c r="D381" s="110"/>
+      <c r="E381" s="117"/>
     </row>
     <row r="382" spans="1:5" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A382" s="111" t="s">
+      <c r="A382" s="118" t="s">
         <v>235</v>
       </c>
-      <c r="B382" s="112"/>
-      <c r="C382" s="112"/>
-      <c r="D382" s="112"/>
-      <c r="E382" s="113"/>
+      <c r="B382" s="119"/>
+      <c r="C382" s="119"/>
+      <c r="D382" s="119"/>
+      <c r="E382" s="120"/>
     </row>
     <row r="383" spans="1:5" s="39" customFormat="1" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A383" s="66" t="s">
@@ -12296,7 +12296,7 @@
         <v>84</v>
       </c>
       <c r="E408" s="40">
-        <v>190</v>
+        <v>209</v>
       </c>
     </row>
     <row r="409" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -12511,13 +12511,13 @@
       <c r="E421" s="61"/>
     </row>
     <row r="422" spans="1:5" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A422" s="111" t="s">
+      <c r="A422" s="118" t="s">
         <v>1302</v>
       </c>
-      <c r="B422" s="112"/>
-      <c r="C422" s="112"/>
-      <c r="D422" s="112"/>
-      <c r="E422" s="113"/>
+      <c r="B422" s="119"/>
+      <c r="C422" s="119"/>
+      <c r="D422" s="119"/>
+      <c r="E422" s="120"/>
     </row>
     <row r="423" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A423" s="66" t="s">
@@ -14454,20 +14454,20 @@
       </c>
     </row>
     <row r="537" spans="1:5" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A537" s="114"/>
-      <c r="B537" s="103"/>
-      <c r="C537" s="103"/>
-      <c r="D537" s="104"/>
-      <c r="E537" s="105"/>
+      <c r="A537" s="116"/>
+      <c r="B537" s="109"/>
+      <c r="C537" s="109"/>
+      <c r="D537" s="110"/>
+      <c r="E537" s="117"/>
     </row>
     <row r="538" spans="1:5" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A538" s="111" t="s">
+      <c r="A538" s="118" t="s">
         <v>338</v>
       </c>
-      <c r="B538" s="112"/>
-      <c r="C538" s="112"/>
-      <c r="D538" s="112"/>
-      <c r="E538" s="113"/>
+      <c r="B538" s="119"/>
+      <c r="C538" s="119"/>
+      <c r="D538" s="119"/>
+      <c r="E538" s="120"/>
     </row>
     <row r="539" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A539" s="66" t="s">
@@ -14825,20 +14825,20 @@
       </c>
     </row>
     <row r="560" spans="1:5" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A560" s="114"/>
-      <c r="B560" s="103"/>
-      <c r="C560" s="103"/>
-      <c r="D560" s="104"/>
-      <c r="E560" s="105"/>
+      <c r="A560" s="116"/>
+      <c r="B560" s="109"/>
+      <c r="C560" s="109"/>
+      <c r="D560" s="110"/>
+      <c r="E560" s="117"/>
     </row>
     <row r="561" spans="1:5" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A561" s="111" t="s">
+      <c r="A561" s="118" t="s">
         <v>353</v>
       </c>
-      <c r="B561" s="112"/>
-      <c r="C561" s="112"/>
-      <c r="D561" s="112"/>
-      <c r="E561" s="113"/>
+      <c r="B561" s="119"/>
+      <c r="C561" s="119"/>
+      <c r="D561" s="119"/>
+      <c r="E561" s="120"/>
     </row>
     <row r="562" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A562" s="66" t="s">
@@ -15451,20 +15451,20 @@
       </c>
     </row>
     <row r="598" spans="1:5" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A598" s="106"/>
-      <c r="B598" s="107"/>
-      <c r="C598" s="107"/>
-      <c r="D598" s="107"/>
-      <c r="E598" s="107"/>
+      <c r="A598" s="128"/>
+      <c r="B598" s="129"/>
+      <c r="C598" s="129"/>
+      <c r="D598" s="129"/>
+      <c r="E598" s="129"/>
     </row>
     <row r="599" spans="1:5" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A599" s="111" t="s">
+      <c r="A599" s="118" t="s">
         <v>370</v>
       </c>
-      <c r="B599" s="112"/>
-      <c r="C599" s="112"/>
-      <c r="D599" s="112"/>
-      <c r="E599" s="113"/>
+      <c r="B599" s="119"/>
+      <c r="C599" s="119"/>
+      <c r="D599" s="119"/>
+      <c r="E599" s="120"/>
     </row>
     <row r="600" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A600" s="66" t="s">
@@ -17457,20 +17457,20 @@
       </c>
     </row>
     <row r="717" spans="1:5" s="39" customFormat="1" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A717" s="114"/>
-      <c r="B717" s="103"/>
-      <c r="C717" s="103"/>
-      <c r="D717" s="104"/>
-      <c r="E717" s="105"/>
+      <c r="A717" s="116"/>
+      <c r="B717" s="109"/>
+      <c r="C717" s="109"/>
+      <c r="D717" s="110"/>
+      <c r="E717" s="117"/>
     </row>
     <row r="718" spans="1:5" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A718" s="111" t="s">
+      <c r="A718" s="118" t="s">
         <v>420</v>
       </c>
-      <c r="B718" s="112"/>
-      <c r="C718" s="112"/>
-      <c r="D718" s="112"/>
-      <c r="E718" s="113"/>
+      <c r="B718" s="119"/>
+      <c r="C718" s="119"/>
+      <c r="D718" s="119"/>
+      <c r="E718" s="120"/>
     </row>
     <row r="719" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A719" s="66" t="s">
@@ -17648,13 +17648,13 @@
       <c r="E729" s="61"/>
     </row>
     <row r="730" spans="1:5" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A730" s="111" t="s">
+      <c r="A730" s="118" t="s">
         <v>1303</v>
       </c>
-      <c r="B730" s="112"/>
-      <c r="C730" s="112"/>
-      <c r="D730" s="112"/>
-      <c r="E730" s="113"/>
+      <c r="B730" s="119"/>
+      <c r="C730" s="119"/>
+      <c r="D730" s="119"/>
+      <c r="E730" s="120"/>
     </row>
     <row r="731" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A731" s="72" t="s">
@@ -17776,20 +17776,20 @@
       </c>
     </row>
     <row r="738" spans="1:5" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A738" s="102"/>
-      <c r="B738" s="103"/>
-      <c r="C738" s="103"/>
-      <c r="D738" s="104"/>
-      <c r="E738" s="105"/>
+      <c r="A738" s="121"/>
+      <c r="B738" s="109"/>
+      <c r="C738" s="109"/>
+      <c r="D738" s="110"/>
+      <c r="E738" s="117"/>
     </row>
     <row r="739" spans="1:5" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A739" s="111" t="s">
+      <c r="A739" s="118" t="s">
         <v>421</v>
       </c>
-      <c r="B739" s="112"/>
-      <c r="C739" s="112"/>
-      <c r="D739" s="112"/>
-      <c r="E739" s="113"/>
+      <c r="B739" s="119"/>
+      <c r="C739" s="119"/>
+      <c r="D739" s="119"/>
+      <c r="E739" s="120"/>
     </row>
     <row r="740" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A740" s="66" t="s">
@@ -17943,20 +17943,20 @@
       </c>
     </row>
     <row r="749" spans="1:5" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A749" s="102"/>
-      <c r="B749" s="103"/>
-      <c r="C749" s="103"/>
-      <c r="D749" s="104"/>
-      <c r="E749" s="105"/>
+      <c r="A749" s="121"/>
+      <c r="B749" s="109"/>
+      <c r="C749" s="109"/>
+      <c r="D749" s="110"/>
+      <c r="E749" s="117"/>
     </row>
     <row r="750" spans="1:5" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A750" s="111" t="s">
+      <c r="A750" s="118" t="s">
         <v>1301</v>
       </c>
-      <c r="B750" s="112"/>
-      <c r="C750" s="112"/>
-      <c r="D750" s="112"/>
-      <c r="E750" s="113"/>
+      <c r="B750" s="119"/>
+      <c r="C750" s="119"/>
+      <c r="D750" s="119"/>
+      <c r="E750" s="120"/>
     </row>
     <row r="751" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A751" s="66" t="s">
@@ -18386,13 +18386,13 @@
       <c r="E775" s="98"/>
     </row>
     <row r="776" spans="1:5" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A776" s="108" t="s">
+      <c r="A776" s="130" t="s">
         <v>1287</v>
       </c>
-      <c r="B776" s="109"/>
-      <c r="C776" s="109"/>
-      <c r="D776" s="109"/>
-      <c r="E776" s="110"/>
+      <c r="B776" s="131"/>
+      <c r="C776" s="131"/>
+      <c r="D776" s="131"/>
+      <c r="E776" s="132"/>
     </row>
     <row r="777" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A777" s="66" t="s">
@@ -20354,13 +20354,13 @@
       <c r="E893" s="100"/>
     </row>
     <row r="894" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A894" s="121" t="s">
+      <c r="A894" s="102" t="s">
         <v>1288</v>
       </c>
-      <c r="B894" s="122"/>
-      <c r="C894" s="122"/>
-      <c r="D894" s="122"/>
-      <c r="E894" s="123"/>
+      <c r="B894" s="103"/>
+      <c r="C894" s="103"/>
+      <c r="D894" s="103"/>
+      <c r="E894" s="104"/>
     </row>
     <row r="895" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A895" s="87" t="s">
@@ -20427,7 +20427,7 @@
         <v>412</v>
       </c>
       <c r="E898" s="48">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="899" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -20444,7 +20444,7 @@
         <v>15</v>
       </c>
       <c r="E899" s="48">
-        <v>252</v>
+        <v>276</v>
       </c>
     </row>
     <row r="900" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -20461,7 +20461,7 @@
         <v>412</v>
       </c>
       <c r="E900" s="48">
-        <v>57</v>
+        <v>62.5</v>
       </c>
     </row>
     <row r="901" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -20478,7 +20478,7 @@
         <v>15</v>
       </c>
       <c r="E901" s="48">
-        <v>540</v>
+        <v>582</v>
       </c>
     </row>
     <row r="902" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -20495,7 +20495,7 @@
         <v>412</v>
       </c>
       <c r="E902" s="48">
-        <v>70</v>
+        <v>76.5</v>
       </c>
     </row>
     <row r="903" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -20512,7 +20512,7 @@
         <v>15</v>
       </c>
       <c r="E903" s="48">
-        <v>660</v>
+        <v>714.5</v>
       </c>
     </row>
     <row r="904" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -20529,7 +20529,7 @@
         <v>412</v>
       </c>
       <c r="E904" s="48">
-        <v>62.5</v>
+        <v>68</v>
       </c>
     </row>
     <row r="905" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -20546,7 +20546,7 @@
         <v>15</v>
       </c>
       <c r="E905" s="48">
-        <v>582</v>
+        <v>636</v>
       </c>
     </row>
     <row r="906" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -20563,7 +20563,7 @@
         <v>412</v>
       </c>
       <c r="E906" s="48">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="907" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -20580,7 +20580,7 @@
         <v>15</v>
       </c>
       <c r="E907" s="48">
-        <v>168</v>
+        <v>186</v>
       </c>
     </row>
     <row r="908" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -20597,7 +20597,7 @@
         <v>412</v>
       </c>
       <c r="E908" s="48">
-        <v>105</v>
+        <v>115</v>
       </c>
     </row>
     <row r="909" spans="1:5" ht="15.75" x14ac:dyDescent="0.2">
@@ -20614,7 +20614,7 @@
         <v>15</v>
       </c>
       <c r="E909" s="48">
-        <v>996</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="910" spans="1:5" ht="15.75" x14ac:dyDescent="0.2"/>
@@ -20633,6 +20633,27 @@
     </row>
   </sheetData>
   <mergeCells count="37">
+    <mergeCell ref="A738:E738"/>
+    <mergeCell ref="A598:E598"/>
+    <mergeCell ref="A214:E214"/>
+    <mergeCell ref="A128:E128"/>
+    <mergeCell ref="A776:E776"/>
+    <mergeCell ref="A730:E730"/>
+    <mergeCell ref="A749:E749"/>
+    <mergeCell ref="A750:E750"/>
+    <mergeCell ref="A537:E537"/>
+    <mergeCell ref="A561:E561"/>
+    <mergeCell ref="A109:E109"/>
+    <mergeCell ref="A538:E538"/>
+    <mergeCell ref="A8:E8"/>
+    <mergeCell ref="A9:E9"/>
+    <mergeCell ref="A129:E129"/>
+    <mergeCell ref="A422:E422"/>
+    <mergeCell ref="A382:E382"/>
+    <mergeCell ref="A110:E110"/>
+    <mergeCell ref="A381:E381"/>
+    <mergeCell ref="A140:E140"/>
+    <mergeCell ref="A215:E215"/>
     <mergeCell ref="A894:E894"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A6:E6"/>
@@ -20649,27 +20670,6 @@
     <mergeCell ref="A560:E560"/>
     <mergeCell ref="A717:E717"/>
     <mergeCell ref="A288:E288"/>
-    <mergeCell ref="A109:E109"/>
-    <mergeCell ref="A538:E538"/>
-    <mergeCell ref="A8:E8"/>
-    <mergeCell ref="A9:E9"/>
-    <mergeCell ref="A129:E129"/>
-    <mergeCell ref="A422:E422"/>
-    <mergeCell ref="A382:E382"/>
-    <mergeCell ref="A110:E110"/>
-    <mergeCell ref="A381:E381"/>
-    <mergeCell ref="A140:E140"/>
-    <mergeCell ref="A215:E215"/>
-    <mergeCell ref="A738:E738"/>
-    <mergeCell ref="A598:E598"/>
-    <mergeCell ref="A214:E214"/>
-    <mergeCell ref="A128:E128"/>
-    <mergeCell ref="A776:E776"/>
-    <mergeCell ref="A730:E730"/>
-    <mergeCell ref="A749:E749"/>
-    <mergeCell ref="A750:E750"/>
-    <mergeCell ref="A537:E537"/>
-    <mergeCell ref="A561:E561"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A4" r:id="rId1" display="mailto:E-mailastralalimentos@gmail.com" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
@@ -20709,78 +20709,78 @@
       <c r="A2" s="148" t="s">
         <v>484</v>
       </c>
-      <c r="B2" s="135"/>
-      <c r="C2" s="136"/>
-      <c r="D2" s="137"/>
-      <c r="E2" s="139"/>
+      <c r="B2" s="134"/>
+      <c r="C2" s="135"/>
+      <c r="D2" s="136"/>
+      <c r="E2" s="138"/>
     </row>
     <row r="3" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="150" t="s">
+      <c r="A3" s="137" t="s">
         <v>485</v>
       </c>
-      <c r="B3" s="135"/>
-      <c r="C3" s="136"/>
-      <c r="D3" s="137"/>
-      <c r="E3" s="139"/>
+      <c r="B3" s="134"/>
+      <c r="C3" s="135"/>
+      <c r="D3" s="136"/>
+      <c r="E3" s="138"/>
     </row>
     <row r="4" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="138" t="s">
+      <c r="A4" s="149" t="s">
         <v>486</v>
       </c>
-      <c r="B4" s="135"/>
-      <c r="C4" s="136"/>
-      <c r="D4" s="137"/>
-      <c r="E4" s="139"/>
+      <c r="B4" s="134"/>
+      <c r="C4" s="135"/>
+      <c r="D4" s="136"/>
+      <c r="E4" s="138"/>
     </row>
     <row r="5" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="150" t="s">
+      <c r="A5" s="137" t="s">
         <v>487</v>
       </c>
-      <c r="B5" s="135"/>
-      <c r="C5" s="136"/>
-      <c r="D5" s="137"/>
-      <c r="E5" s="139"/>
+      <c r="B5" s="134"/>
+      <c r="C5" s="135"/>
+      <c r="D5" s="136"/>
+      <c r="E5" s="138"/>
     </row>
     <row r="6" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="144"/>
-      <c r="B6" s="135"/>
-      <c r="C6" s="136"/>
-      <c r="D6" s="137"/>
-      <c r="E6" s="139"/>
+      <c r="B6" s="134"/>
+      <c r="C6" s="135"/>
+      <c r="D6" s="136"/>
+      <c r="E6" s="138"/>
     </row>
     <row r="7" spans="1:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="147" t="s">
         <v>488</v>
       </c>
-      <c r="B7" s="135"/>
-      <c r="C7" s="136"/>
-      <c r="D7" s="137"/>
-      <c r="E7" s="139"/>
+      <c r="B7" s="134"/>
+      <c r="C7" s="135"/>
+      <c r="D7" s="136"/>
+      <c r="E7" s="138"/>
     </row>
     <row r="8" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="145" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="135"/>
-      <c r="C8" s="136"/>
-      <c r="D8" s="137"/>
-      <c r="E8" s="139"/>
+      <c r="B8" s="134"/>
+      <c r="C8" s="135"/>
+      <c r="D8" s="136"/>
+      <c r="E8" s="138"/>
     </row>
     <row r="9" spans="1:7" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="146"/>
-      <c r="B9" s="135"/>
-      <c r="C9" s="136"/>
-      <c r="D9" s="137"/>
-      <c r="E9" s="139"/>
+      <c r="B9" s="134"/>
+      <c r="C9" s="135"/>
+      <c r="D9" s="136"/>
+      <c r="E9" s="138"/>
     </row>
     <row r="10" spans="1:7" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="140" t="s">
+      <c r="A10" s="150" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="112"/>
-      <c r="C10" s="112"/>
-      <c r="D10" s="112"/>
-      <c r="E10" s="113"/>
+      <c r="B10" s="119"/>
+      <c r="C10" s="119"/>
+      <c r="D10" s="119"/>
+      <c r="E10" s="120"/>
     </row>
     <row r="11" spans="1:7" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="31" t="s">
@@ -22503,19 +22503,19 @@
       </c>
     </row>
     <row r="112" spans="1:5" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A112" s="134"/>
-      <c r="B112" s="135"/>
-      <c r="C112" s="136"/>
-      <c r="D112" s="137"/>
+      <c r="A112" s="133"/>
+      <c r="B112" s="134"/>
+      <c r="C112" s="135"/>
+      <c r="D112" s="136"/>
       <c r="E112" s="25"/>
     </row>
     <row r="113" spans="1:5" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A113" s="149" t="s">
+      <c r="A113" s="140" t="s">
         <v>86</v>
       </c>
-      <c r="B113" s="112"/>
-      <c r="C113" s="112"/>
-      <c r="D113" s="120"/>
+      <c r="B113" s="119"/>
+      <c r="C113" s="119"/>
+      <c r="D113" s="127"/>
       <c r="E113" s="28"/>
     </row>
     <row r="114" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -22808,19 +22808,19 @@
       </c>
     </row>
     <row r="131" spans="1:5" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A131" s="134"/>
-      <c r="B131" s="135"/>
-      <c r="C131" s="136"/>
-      <c r="D131" s="137"/>
+      <c r="A131" s="133"/>
+      <c r="B131" s="134"/>
+      <c r="C131" s="135"/>
+      <c r="D131" s="136"/>
       <c r="E131" s="25"/>
     </row>
     <row r="132" spans="1:5" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A132" s="149" t="s">
+      <c r="A132" s="140" t="s">
         <v>95</v>
       </c>
-      <c r="B132" s="112"/>
-      <c r="C132" s="112"/>
-      <c r="D132" s="120"/>
+      <c r="B132" s="119"/>
+      <c r="C132" s="119"/>
+      <c r="D132" s="127"/>
       <c r="E132" s="28"/>
     </row>
     <row r="133" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -22994,19 +22994,19 @@
       </c>
     </row>
     <row r="143" spans="1:5" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A143" s="134"/>
-      <c r="B143" s="135"/>
-      <c r="C143" s="136"/>
-      <c r="D143" s="137"/>
+      <c r="A143" s="133"/>
+      <c r="B143" s="134"/>
+      <c r="C143" s="135"/>
+      <c r="D143" s="136"/>
       <c r="E143" s="25"/>
     </row>
     <row r="144" spans="1:5" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A144" s="149" t="s">
+      <c r="A144" s="140" t="s">
         <v>106</v>
       </c>
-      <c r="B144" s="112"/>
-      <c r="C144" s="112"/>
-      <c r="D144" s="120"/>
+      <c r="B144" s="119"/>
+      <c r="C144" s="119"/>
+      <c r="D144" s="127"/>
       <c r="E144" s="28"/>
     </row>
     <row r="145" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -23639,19 +23639,19 @@
       </c>
     </row>
     <row r="182" spans="1:5" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A182" s="134"/>
-      <c r="B182" s="135"/>
-      <c r="C182" s="136"/>
-      <c r="D182" s="137"/>
+      <c r="A182" s="133"/>
+      <c r="B182" s="134"/>
+      <c r="C182" s="135"/>
+      <c r="D182" s="136"/>
       <c r="E182" s="25"/>
     </row>
     <row r="183" spans="1:5" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A183" s="133" t="s">
+      <c r="A183" s="139" t="s">
         <v>148</v>
       </c>
-      <c r="B183" s="112"/>
-      <c r="C183" s="112"/>
-      <c r="D183" s="112"/>
+      <c r="B183" s="119"/>
+      <c r="C183" s="119"/>
+      <c r="D183" s="119"/>
       <c r="E183" s="26"/>
     </row>
     <row r="184" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -24513,19 +24513,19 @@
       </c>
     </row>
     <row r="241" spans="1:5" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A241" s="134"/>
-      <c r="B241" s="135"/>
-      <c r="C241" s="136"/>
-      <c r="D241" s="137"/>
+      <c r="A241" s="133"/>
+      <c r="B241" s="134"/>
+      <c r="C241" s="135"/>
+      <c r="D241" s="136"/>
       <c r="E241" s="25"/>
     </row>
     <row r="242" spans="1:5" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A242" s="133" t="s">
+      <c r="A242" s="139" t="s">
         <v>186</v>
       </c>
-      <c r="B242" s="112"/>
-      <c r="C242" s="112"/>
-      <c r="D242" s="112"/>
+      <c r="B242" s="119"/>
+      <c r="C242" s="119"/>
+      <c r="D242" s="119"/>
       <c r="E242" s="28"/>
     </row>
     <row r="243" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -25746,21 +25746,21 @@
       </c>
     </row>
     <row r="324" spans="1:8" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A324" s="134"/>
-      <c r="B324" s="135"/>
-      <c r="C324" s="136"/>
-      <c r="D324" s="137"/>
+      <c r="A324" s="133"/>
+      <c r="B324" s="134"/>
+      <c r="C324" s="135"/>
+      <c r="D324" s="136"/>
       <c r="E324" s="25"/>
       <c r="G324" s="30"/>
       <c r="H324" s="30"/>
     </row>
     <row r="325" spans="1:8" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A325" s="133" t="s">
+      <c r="A325" s="139" t="s">
         <v>235</v>
       </c>
-      <c r="B325" s="112"/>
-      <c r="C325" s="112"/>
-      <c r="D325" s="112"/>
+      <c r="B325" s="119"/>
+      <c r="C325" s="119"/>
+      <c r="D325" s="119"/>
       <c r="E325" s="28"/>
     </row>
     <row r="326" spans="1:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -26257,19 +26257,19 @@
       </c>
     </row>
     <row r="355" spans="1:5" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A355" s="134"/>
-      <c r="B355" s="135"/>
-      <c r="C355" s="136"/>
-      <c r="D355" s="137"/>
+      <c r="A355" s="133"/>
+      <c r="B355" s="134"/>
+      <c r="C355" s="135"/>
+      <c r="D355" s="136"/>
       <c r="E355" s="25"/>
     </row>
     <row r="356" spans="1:5" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A356" s="133" t="s">
+      <c r="A356" s="139" t="s">
         <v>261</v>
       </c>
-      <c r="B356" s="112"/>
-      <c r="C356" s="112"/>
-      <c r="D356" s="112"/>
+      <c r="B356" s="119"/>
+      <c r="C356" s="119"/>
+      <c r="D356" s="119"/>
       <c r="E356" s="28"/>
     </row>
     <row r="357" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -28024,19 +28024,19 @@
       </c>
     </row>
     <row r="460" spans="1:5" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A460" s="134"/>
-      <c r="B460" s="135"/>
-      <c r="C460" s="136"/>
-      <c r="D460" s="137"/>
+      <c r="A460" s="133"/>
+      <c r="B460" s="134"/>
+      <c r="C460" s="135"/>
+      <c r="D460" s="136"/>
       <c r="E460" s="25"/>
     </row>
     <row r="461" spans="1:5" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A461" s="133" t="s">
+      <c r="A461" s="139" t="s">
         <v>338</v>
       </c>
-      <c r="B461" s="112"/>
-      <c r="C461" s="112"/>
-      <c r="D461" s="112"/>
+      <c r="B461" s="119"/>
+      <c r="C461" s="119"/>
+      <c r="D461" s="119"/>
       <c r="E461" s="28"/>
     </row>
     <row r="462" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -28329,19 +28329,19 @@
       </c>
     </row>
     <row r="479" spans="1:5" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A479" s="134"/>
-      <c r="B479" s="135"/>
-      <c r="C479" s="136"/>
-      <c r="D479" s="137"/>
+      <c r="A479" s="133"/>
+      <c r="B479" s="134"/>
+      <c r="C479" s="135"/>
+      <c r="D479" s="136"/>
       <c r="E479" s="25"/>
     </row>
     <row r="480" spans="1:5" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A480" s="133" t="s">
+      <c r="A480" s="139" t="s">
         <v>353</v>
       </c>
-      <c r="B480" s="112"/>
-      <c r="C480" s="112"/>
-      <c r="D480" s="112"/>
+      <c r="B480" s="119"/>
+      <c r="C480" s="119"/>
+      <c r="D480" s="119"/>
       <c r="E480" s="28"/>
     </row>
     <row r="481" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -28770,19 +28770,19 @@
       </c>
     </row>
     <row r="506" spans="1:5" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A506" s="134"/>
-      <c r="B506" s="135"/>
-      <c r="C506" s="136"/>
-      <c r="D506" s="137"/>
+      <c r="A506" s="133"/>
+      <c r="B506" s="134"/>
+      <c r="C506" s="135"/>
+      <c r="D506" s="136"/>
       <c r="E506" s="25"/>
     </row>
     <row r="507" spans="1:5" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A507" s="133" t="s">
+      <c r="A507" s="139" t="s">
         <v>370</v>
       </c>
-      <c r="B507" s="112"/>
-      <c r="C507" s="112"/>
-      <c r="D507" s="112"/>
+      <c r="B507" s="119"/>
+      <c r="C507" s="119"/>
+      <c r="D507" s="119"/>
       <c r="E507" s="28"/>
     </row>
     <row r="508" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -30297,19 +30297,19 @@
       </c>
     </row>
     <row r="597" spans="1:7" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A597" s="134"/>
-      <c r="B597" s="135"/>
-      <c r="C597" s="136"/>
-      <c r="D597" s="137"/>
+      <c r="A597" s="133"/>
+      <c r="B597" s="134"/>
+      <c r="C597" s="135"/>
+      <c r="D597" s="136"/>
       <c r="E597" s="25"/>
     </row>
     <row r="598" spans="1:7" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A598" s="133" t="s">
+      <c r="A598" s="139" t="s">
         <v>420</v>
       </c>
-      <c r="B598" s="112"/>
-      <c r="C598" s="112"/>
-      <c r="D598" s="112"/>
+      <c r="B598" s="119"/>
+      <c r="C598" s="119"/>
+      <c r="D598" s="119"/>
       <c r="E598" s="28"/>
     </row>
     <row r="599" spans="1:7" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -30449,20 +30449,20 @@
       </c>
     </row>
     <row r="607" spans="1:7" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A607" s="134"/>
-      <c r="B607" s="135"/>
-      <c r="C607" s="136"/>
-      <c r="D607" s="137"/>
+      <c r="A607" s="133"/>
+      <c r="B607" s="134"/>
+      <c r="C607" s="135"/>
+      <c r="D607" s="136"/>
       <c r="E607" s="25"/>
       <c r="G607" s="29"/>
     </row>
     <row r="608" spans="1:7" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A608" s="133" t="s">
+      <c r="A608" s="139" t="s">
         <v>421</v>
       </c>
-      <c r="B608" s="112"/>
-      <c r="C608" s="112"/>
-      <c r="D608" s="112"/>
+      <c r="B608" s="119"/>
+      <c r="C608" s="119"/>
+      <c r="D608" s="119"/>
       <c r="E608" s="27"/>
     </row>
     <row r="609" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -30551,19 +30551,19 @@
       </c>
     </row>
     <row r="614" spans="1:5" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A614" s="134"/>
-      <c r="B614" s="135"/>
-      <c r="C614" s="136"/>
-      <c r="D614" s="137"/>
+      <c r="A614" s="133"/>
+      <c r="B614" s="134"/>
+      <c r="C614" s="135"/>
+      <c r="D614" s="136"/>
       <c r="E614" s="25"/>
     </row>
     <row r="615" spans="1:5" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A615" s="133" t="s">
+      <c r="A615" s="139" t="s">
         <v>422</v>
       </c>
-      <c r="B615" s="112"/>
-      <c r="C615" s="112"/>
-      <c r="D615" s="112"/>
+      <c r="B615" s="119"/>
+      <c r="C615" s="119"/>
+      <c r="D615" s="119"/>
       <c r="E615" s="28"/>
     </row>
     <row r="616" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -31928,25 +31928,6 @@
     </row>
   </sheetData>
   <mergeCells count="35">
-    <mergeCell ref="A597:D597"/>
-    <mergeCell ref="A506:D506"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A598:D598"/>
-    <mergeCell ref="A132:D132"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A460:D460"/>
-    <mergeCell ref="A112:D112"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A8:E9"/>
-    <mergeCell ref="A7:E7"/>
-    <mergeCell ref="A143:D143"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A113:D113"/>
-    <mergeCell ref="A242:D242"/>
-    <mergeCell ref="A144:D144"/>
-    <mergeCell ref="A131:D131"/>
-    <mergeCell ref="A324:D324"/>
-    <mergeCell ref="A3:E3"/>
     <mergeCell ref="A615:D615"/>
     <mergeCell ref="A182:D182"/>
     <mergeCell ref="A480:D480"/>
@@ -31963,6 +31944,25 @@
     <mergeCell ref="A607:D607"/>
     <mergeCell ref="A608:D608"/>
     <mergeCell ref="A507:D507"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A460:D460"/>
+    <mergeCell ref="A112:D112"/>
+    <mergeCell ref="A6:E6"/>
+    <mergeCell ref="A8:E9"/>
+    <mergeCell ref="A7:E7"/>
+    <mergeCell ref="A143:D143"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A113:D113"/>
+    <mergeCell ref="A242:D242"/>
+    <mergeCell ref="A144:D144"/>
+    <mergeCell ref="A131:D131"/>
+    <mergeCell ref="A324:D324"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A597:D597"/>
+    <mergeCell ref="A506:D506"/>
+    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="A598:D598"/>
+    <mergeCell ref="A132:D132"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A4" r:id="rId1" display="mailto:E-mailastralalimentos@gmail.com" xr:uid="{00000000-0004-0000-0100-000000000000}"/>

</xml_diff>